<commit_message>
WS5: review fixes - plan defaults per key, per-key inherited references, formula bounds, spec hash check, missing Benefits, renamed sheets, negative benefits
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CEPjX4ZK9rqa23wykfCmQq
</commit_message>
<xml_diff>
--- a/fixtures/C_ALPHA/cedant_workbook.xlsx
+++ b/fixtures/C_ALPHA/cedant_workbook.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4986" uniqueCount="2430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4988" uniqueCount="2432">
   <si>
     <t>INDIVIDUAL - RGN_A</t>
   </si>
@@ -7270,6 +7270,12 @@
   </si>
   <si>
     <t>4d971354e45b809b7311558a4b3068bde6fe30e9403d9f80b8c77ad7f7e0d769</t>
+  </si>
+  <si>
+    <t>cedant_spec_hash</t>
+  </si>
+  <si>
+    <t>97b7356383303a8b9492eff451d9b9eb7c78afbb31a9dffb0100437f50ea26bb</t>
   </si>
   <si>
     <t>template_spec_version</t>
@@ -32341,7 +32347,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -32448,6 +32454,14 @@
         <v>2429</v>
       </c>
     </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>2430</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2431</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>